<commit_message>
Fixed compatibility issues: Made xarray and h5netcdf example optional as they are third party packages Adjusted label formatting - fixed r-strings for $\pi$ labeling Legend location: Changed "outside center" to "upper center" as "outside" is not actually a keyword for matplotlib, but seems to sometimes work. Added non-comboplot low temperature plot case in CIII example Added more descriptions and comments in the example headers.
</commit_message>
<xml_diff>
--- a/ExamplesList.xlsx
+++ b/ExamplesList.xlsx
@@ -43,19 +43,19 @@
     <t xml:space="preserve">He</t>
   </si>
   <si>
-    <t xml:space="preserve">Shows polarization filter matching and accurate B-field values. Shows low resolution allows for similar curve to spectrometer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WI_ex1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WI_ex2</t>
+    <t xml:space="preserve">Shows polarization filter matching and accurate B-field values. Shows low resolution allows for similar curve to spectrometer. Shows non dipole-like transitions</t>
   </si>
   <si>
     <t xml:space="preserve">Rb_ex1</t>
   </si>
   <si>
+    <t xml:space="preserve">Demonstrate ability to include hyperfine structure</t>
+  </si>
+  <si>
     <t xml:space="preserve">SpectrometerPredict</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary workhorse example which generates slider plots. Great for predicting if spectral features can be resolved for given temperature, magnetic field, and/or spectrometer resolution.</t>
   </si>
 </sst>
 </file>
@@ -131,8 +131,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -325,64 +333,63 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>